<commit_message>
Powder tags: remove Function_ tags (powders shouldn't be in tea-only By-Function collections); add REPLACE file to strip them from already-tagged products
</commit_message>
<xml_diff>
--- a/matrixify/products-powder-tags.xlsx
+++ b/matrixify/products-powder-tags.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Superfood Blend, Function_Detox</t>
+          <t>Category_Powder, Type_Superfood Blend</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Superfood Blend, Function_Detox</t>
+          <t>Category_Powder, Type_Superfood Blend</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Superfood Blend, Function_Detox</t>
+          <t>Category_Powder, Type_Superfood Blend</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Mushroom Powder, Function_Focus and Energy</t>
+          <t>Category_Powder, Type_Mushroom Powder</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Superfood Blend, Function_Focus and Energy</t>
+          <t>Category_Powder, Type_Superfood Blend</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Mushroom Powder, Function_Immunity</t>
+          <t>Category_Powder, Type_Mushroom Powder</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Mushroom Powder, Function_Focus and Energy</t>
+          <t>Category_Powder, Type_Mushroom Powder</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Superfood Blend, Function_Focus and Energy</t>
+          <t>Category_Powder, Type_Superfood Blend</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Superfood Blend, Function_Wind down</t>
+          <t>Category_Powder, Type_Superfood Blend</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Mushroom Powder, Function_Immunity</t>
+          <t>Category_Powder, Type_Mushroom Powder</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Superfood Blend, Function_Wind down</t>
+          <t>Category_Powder, Type_Superfood Blend</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Category_Powder, Type_Superfood Blend, Function_Focus and Energy</t>
+          <t>Category_Powder, Type_Superfood Blend</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">

</xml_diff>